<commit_message>
Split D4 cause analysis into four A-G merged cells and fix D8 layout.
Pre-expand the xlsx template with four D4 rows for 5-Why, fishbone, association rules, and root cause; merge D8 content across A-G with top-left alignment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/模板1-8D报告.xlsx
+++ b/templates/模板1-8D报告.xlsx
@@ -1000,7 +1000,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1129,6 +1129,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -1204,6 +1213,9 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1561,7 +1573,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="13.75" style="2" customWidth="1"/>
@@ -1803,167 +1815,185 @@
       <c r="F20" s="48"/>
       <c r="G20" s="49"/>
     </row>
-    <row r="21" s="1" customFormat="1" ht="21" customHeight="1" spans="1:9">
+    <row r="21" s="1" customFormat="1" ht="45" customHeight="1" spans="1:9">
       <c r="A21" s="50"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="51" t="s">
-        <v>20</v>
-      </c>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
       <c r="F21" s="51"/>
       <c r="G21" s="52"/>
     </row>
-    <row r="22" s="1" customFormat="1" ht="13.5" spans="1:9">
-      <c r="A22" s="32" t="s">
+    <row r="22" s="1" customFormat="1" ht="45" customHeight="1" spans="1:9">
+      <c r="A22" s="50"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
+    </row>
+    <row r="23" s="1" customFormat="1" ht="21" customHeight="1" spans="1:9">
+      <c r="A23" s="53"/>
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="54" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="54"/>
+      <c r="G23" s="55"/>
+    </row>
+    <row r="24" s="1" customFormat="1" ht="13.5" spans="1:9">
+      <c r="A24" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="53"/>
-    </row>
-    <row r="23" s="1" customFormat="1" ht="83.25" customHeight="1" spans="1:9">
-      <c r="A23" s="54"/>
-      <c r="B23" s="55"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="55"/>
-      <c r="E23" s="55"/>
-      <c r="F23" s="55"/>
-      <c r="G23" s="56"/>
-    </row>
-    <row r="24" s="1" customFormat="1" ht="21.95" customHeight="1" spans="1:9">
-      <c r="A24" s="38"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="57" t="s">
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="56"/>
+    </row>
+    <row r="25" s="1" customFormat="1" ht="83.25" customHeight="1" spans="1:9">
+      <c r="A25" s="57"/>
+      <c r="B25" s="58"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="59"/>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="21.95" customHeight="1" spans="1:9">
+      <c r="A26" s="38"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="57"/>
-      <c r="G24" s="58"/>
-    </row>
-    <row r="25" s="1" customFormat="1" ht="13.5" spans="1:9">
-      <c r="A25" s="32" t="s">
+      <c r="F26" s="60"/>
+      <c r="G26" s="61"/>
+    </row>
+    <row r="27" s="1" customFormat="1" ht="13.5" spans="1:9">
+      <c r="A27" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="59"/>
-      <c r="I25" s="60"/>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="74.25" customHeight="1" spans="1:9">
-      <c r="A26" s="61"/>
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="63"/>
-      <c r="I26" s="60"/>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="23.1" customHeight="1" spans="1:9">
-      <c r="A27" s="64" t="s">
+      <c r="B27" s="33"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="62"/>
+      <c r="I27" s="63"/>
+    </row>
+    <row r="28" s="1" customFormat="1" ht="74.25" customHeight="1" spans="1:9">
+      <c r="A28" s="64"/>
+      <c r="B28" s="65"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="66"/>
+      <c r="I28" s="63"/>
+    </row>
+    <row r="29" s="1" customFormat="1" ht="23.1" customHeight="1" spans="1:9">
+      <c r="A29" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="24"/>
-      <c r="C27" s="65"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="66" t="s">
+      <c r="B29" s="24"/>
+      <c r="C29" s="68"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="F27" s="67" t="s">
+      <c r="F29" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="G27" s="68"/>
-      <c r="I27" s="60"/>
-    </row>
-    <row r="28" s="1" customFormat="1" ht="13.5" spans="1:9">
-      <c r="A28" s="32" t="s">
+      <c r="G29" s="71"/>
+      <c r="I29" s="63"/>
+    </row>
+    <row r="30" s="1" customFormat="1" ht="13.5" spans="1:9">
+      <c r="A30" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="59"/>
-      <c r="I28" s="60"/>
-    </row>
-    <row r="29" s="1" customFormat="1" ht="114.75" customHeight="1" spans="1:9">
-      <c r="A29" s="44"/>
-      <c r="B29" s="45"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
-      <c r="G29" s="46"/>
-      <c r="I29" s="60"/>
-    </row>
-    <row r="30" s="1" customFormat="1" ht="18" customHeight="1" spans="1:9">
-      <c r="A30" s="69"/>
-      <c r="B30" s="70"/>
-      <c r="C30" s="70"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="71" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" s="72" t="s">
-        <v>14</v>
-      </c>
-      <c r="G30" s="68"/>
-    </row>
-    <row r="31" s="1" customFormat="1" ht="13.5" spans="1:9">
-      <c r="A31" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="73"/>
-      <c r="C31" s="73"/>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="74"/>
-    </row>
-    <row r="32" s="1" customFormat="1" ht="18.95" customHeight="1" spans="1:9">
-      <c r="A32" s="17" t="s">
-        <v>13</v>
-      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="62"/>
+      <c r="I30" s="63"/>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="114.75" customHeight="1" spans="1:9">
+      <c r="A31" s="44"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="45"/>
+      <c r="G31" s="46"/>
+      <c r="I31" s="63"/>
+    </row>
+    <row r="32" s="1" customFormat="1" ht="18" customHeight="1" spans="1:9">
+      <c r="A32" s="72"/>
       <c r="B32" s="73"/>
       <c r="C32" s="73"/>
       <c r="D32" s="73"/>
-      <c r="E32" s="73"/>
-      <c r="F32" s="73"/>
-      <c r="G32" s="74"/>
-    </row>
-    <row r="33" s="1" customFormat="1" ht="48" customHeight="1" spans="1:7">
-      <c r="A33" s="23"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="66" t="s">
+      <c r="E32" s="74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="75" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="71"/>
+    </row>
+    <row r="33" s="1" customFormat="1" ht="13.5" spans="1:7">
+      <c r="A33" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="76"/>
+      <c r="C33" s="76"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="77"/>
+    </row>
+    <row r="34" s="1" customFormat="1" ht="18.95" customHeight="1" spans="1:7">
+      <c r="A34" s="78" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="79"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="79"/>
+      <c r="E34" s="79"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="80"/>
+    </row>
+    <row r="35" s="1" customFormat="1" ht="48" customHeight="1" spans="1:7">
+      <c r="A35" s="23"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="G33" s="75"/>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="76" t="s">
+      <c r="G35" s="81"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="82" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="76"/>
-      <c r="C34" s="76"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
+      <c r="B36" s="82"/>
+      <c r="C36" s="82"/>
+      <c r="D36" s="82"/>
+      <c r="E36" s="82"/>
+      <c r="F36" s="82"/>
+      <c r="G36" s="82"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
@@ -1972,12 +2002,15 @@
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="A23:G23"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A3:G4"/>
     <mergeCell ref="A1:G2"/>
     <mergeCell ref="A15:G16"/>
@@ -1987,8 +2020,8 @@
   <pageSetup paperSize="9" scale="90" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0"/>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="27" max="255" man="1"/>
-    <brk id="33" max="255" man="1"/>
+    <brk id="29" max="255" man="1"/>
+    <brk id="35" max="255" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Center fishbone image in D4 cell and unify signature row heights.
Use OneCellAnchor offsets to vertically and horizontally center the fishbone in C:G, and set signature rows R34-R35 to a consistent 30pt height.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/模板1-8D报告.xlsx
+++ b/templates/模板1-8D报告.xlsx
@@ -1181,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col width="13.75" customWidth="1" style="52" min="1" max="1"/>
@@ -1566,7 +1566,7 @@
       <c r="A33" s="72" t="n"/>
       <c r="G33" s="50" t="n"/>
     </row>
-    <row r="34" ht="27" customFormat="1" customHeight="1" s="49">
+    <row r="34" ht="30" customFormat="1" customHeight="1" s="49">
       <c r="A34" s="48" t="inlineStr">
         <is>
           <t>签名：</t>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G34" s="50" t="n"/>
     </row>
-    <row r="35" ht="31.5" customFormat="1" customHeight="1" s="49" thickBot="1">
+    <row r="35" ht="30" customFormat="1" customHeight="1" s="49" thickBot="1">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>

</xml_diff>